<commit_message>
fix(templates): update payroll template file
</commit_message>
<xml_diff>
--- a/apps/sis-laravel/public/templates/PAYROLL_TEMPLATE.xlsx
+++ b/apps/sis-laravel/public/templates/PAYROLL_TEMPLATE.xlsx
@@ -125,7 +125,7 @@
     <t>MA. TERESITA D. MACAPAGAL</t>
   </si>
   <si>
-    <t>FREDIZ B. DAQUILA</t>
+    <t>GRACE G. GUZMAN</t>
   </si>
   <si>
     <t>JOSEL F. VIOLAGO</t>
@@ -134,7 +134,7 @@
     <t>City Administrator</t>
   </si>
   <si>
-    <t xml:space="preserve">                        Name &amp; Signature of City Accountant</t>
+    <t xml:space="preserve">           Accountant IV &amp; Acting City Accountant</t>
   </si>
   <si>
     <t>Name &amp; Signature of Officer</t>
@@ -149,7 +149,7 @@
     <t>ARNOLD A. ESCUADRO</t>
   </si>
   <si>
-    <t>Name &amp; Signature of Treasurer</t>
+    <t>CityTreasurer</t>
   </si>
   <si>
     <t>CERTIFIED:Each employee whose appears above has</t>

</xml_diff>